<commit_message>
Data: Update official Fang DEDP crude oil production figures (Jan-Jul 2569)
</commit_message>
<xml_diff>
--- a/fang_production_master.xlsx
+++ b/fang_production_master.xlsx
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>594.9029032257999</v>
       </c>
     </row>
     <row r="3">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>618.93928571428</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>637.31709677419</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>651.3546666</v>
       </c>
     </row>
     <row r="6">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>628.89258064516</v>
       </c>
     </row>
     <row r="7">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>610.4</v>
+        <v>610.355666666</v>
       </c>
     </row>
     <row r="8">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>618.47548387096</v>
       </c>
     </row>
     <row r="9">
@@ -929,13 +929,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{881856D5-BB0A-493E-817C-9D269A98F2D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F62F021A-9190-4141-ADC0-87B4E7103B37}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92DE5CFE-BAE4-4815-B873-FD9DBC98B6E3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{622C67E4-2A77-45BF-B235-AD27C787BB90}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5DDCE23-3609-41BC-927C-0C2607FA2AB9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB11A42B-19DB-4E2B-A076-C8F31C78F36F}"/>
 </file>
</xml_diff>